<commit_message>
data(Gerencia): actualizar Excel/CSV y soporte de ventas grandes (oficial y pruebas)
Republica en la web (oficial/ y pruebas/) los mismos cambios ya subidos
al repo privado (commit 254ba80 de develop): INVENTARIO.xlsx, INVENTARIO
POR MESES.xlsx, TABLERO.xlsx, TALENTO HUMANO.xlsx, VENTAS.csv actualizados,
mas dias-inventario.html y jszip.min.js para leer archivos de ventas
grandes en streaming.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/oficial/Gerencia/TALENTO HUMANO.xlsx
+++ b/oficial/Gerencia/TALENTO HUMANO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/APP OPAUSTRO/APP OPAUSTRO/Gerencia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{996977CD-B87C-4485-A8E4-AA98CA6C457C}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{674EB762-6582-42B0-8157-783A31CCBF6F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TALENTO ACTUAL" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="78">
   <si>
     <t>TALENTO HUMANO - SITUACION ACTUAL POR DEPARTAMENTO</t>
   </si>
@@ -266,6 +266,9 @@
   </si>
   <si>
     <t>Adulteracion de recibo de cobro</t>
+  </si>
+  <si>
+    <t>AGOSTO</t>
   </si>
 </sst>
 </file>
@@ -838,7 +841,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="16">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="C4" s="4">
         <v>79</v>
@@ -881,7 +884,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="16">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="C5" s="4">
         <v>22</v>
@@ -924,7 +927,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="16">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="C6" s="4">
         <v>29</v>
@@ -1020,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1893,6 +1896,120 @@
       </c>
       <c r="K24" s="13">
         <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="11">
+        <v>75</v>
+      </c>
+      <c r="E25" s="11">
+        <v>4</v>
+      </c>
+      <c r="F25" s="11">
+        <v>5</v>
+      </c>
+      <c r="G25" s="11">
+        <v>0</v>
+      </c>
+      <c r="H25" s="11">
+        <v>0</v>
+      </c>
+      <c r="I25" s="13">
+        <f t="shared" ref="I25:I27" si="9">IF(D25=0,0,(E25+F25)/D25)</f>
+        <v>0.12</v>
+      </c>
+      <c r="J25" s="13">
+        <f t="shared" ref="J25:J27" si="10">IF(D25=0,0,E25/D25)</f>
+        <v>5.3333333333333337E-2</v>
+      </c>
+      <c r="K25" s="13">
+        <f t="shared" ref="K25:K27" si="11">IF(D25=0,0,F25/D25)</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="11">
+        <v>22</v>
+      </c>
+      <c r="E26" s="11">
+        <v>0</v>
+      </c>
+      <c r="F26" s="11">
+        <v>0</v>
+      </c>
+      <c r="G26" s="11">
+        <v>0</v>
+      </c>
+      <c r="H26" s="11">
+        <v>0</v>
+      </c>
+      <c r="I26" s="13">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J26" s="13">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="K26" s="13">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="11">
+        <v>29</v>
+      </c>
+      <c r="E27" s="11">
+        <v>0</v>
+      </c>
+      <c r="F27" s="11">
+        <v>0</v>
+      </c>
+      <c r="G27" s="11">
+        <v>0</v>
+      </c>
+      <c r="H27" s="11">
+        <v>0</v>
+      </c>
+      <c r="I27" s="13">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="13">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="K27" s="13">
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(oficial): restaurar oficial/ al contenido de main privado (OFICIAL)
Entre el 18-09 y el 23-09 se publicaron en oficial/ archivos tomados de
develop (pruebas), dejando Login y Admin (control_usuarios,
control_modulos) apuntando a los Apps Script de pruebas. Se restaura
oficial/ archivo por archivo desde main del repo privado (177c547,
v1.0.16): endpoints, paginas de Gerencia y archivos de datos.
Se eliminan BALANCE.xlsx y jszip.min.js (no existen en main).
pruebas/ no se modifica.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/oficial/Gerencia/TALENTO HUMANO.xlsx
+++ b/oficial/Gerencia/TALENTO HUMANO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/APP OPAUSTRO/APP OPAUSTRO/Gerencia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{674EB762-6582-42B0-8157-783A31CCBF6F}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{996977CD-B87C-4485-A8E4-AA98CA6C457C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TALENTO ACTUAL" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="77">
   <si>
     <t>TALENTO HUMANO - SITUACION ACTUAL POR DEPARTAMENTO</t>
   </si>
@@ -266,9 +266,6 @@
   </si>
   <si>
     <t>Adulteracion de recibo de cobro</t>
-  </si>
-  <si>
-    <t>AGOSTO</t>
   </si>
 </sst>
 </file>
@@ -841,7 +838,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="16">
-        <v>46265</v>
+        <v>46234</v>
       </c>
       <c r="C4" s="4">
         <v>79</v>
@@ -884,7 +881,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="16">
-        <v>46265</v>
+        <v>46234</v>
       </c>
       <c r="C5" s="4">
         <v>22</v>
@@ -927,7 +924,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="16">
-        <v>46265</v>
+        <v>46234</v>
       </c>
       <c r="C6" s="4">
         <v>29</v>
@@ -1023,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1896,120 +1893,6 @@
       </c>
       <c r="K24" s="13">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="11">
-        <v>2026</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D25" s="11">
-        <v>75</v>
-      </c>
-      <c r="E25" s="11">
-        <v>4</v>
-      </c>
-      <c r="F25" s="11">
-        <v>5</v>
-      </c>
-      <c r="G25" s="11">
-        <v>0</v>
-      </c>
-      <c r="H25" s="11">
-        <v>0</v>
-      </c>
-      <c r="I25" s="13">
-        <f t="shared" ref="I25:I27" si="9">IF(D25=0,0,(E25+F25)/D25)</f>
-        <v>0.12</v>
-      </c>
-      <c r="J25" s="13">
-        <f t="shared" ref="J25:J27" si="10">IF(D25=0,0,E25/D25)</f>
-        <v>5.3333333333333337E-2</v>
-      </c>
-      <c r="K25" s="13">
-        <f t="shared" ref="K25:K27" si="11">IF(D25=0,0,F25/D25)</f>
-        <v>6.6666666666666666E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="11">
-        <v>2026</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D26" s="11">
-        <v>22</v>
-      </c>
-      <c r="E26" s="11">
-        <v>0</v>
-      </c>
-      <c r="F26" s="11">
-        <v>0</v>
-      </c>
-      <c r="G26" s="11">
-        <v>0</v>
-      </c>
-      <c r="H26" s="11">
-        <v>0</v>
-      </c>
-      <c r="I26" s="13">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J26" s="13">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="K26" s="13">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="11">
-        <v>2026</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D27" s="11">
-        <v>29</v>
-      </c>
-      <c r="E27" s="11">
-        <v>0</v>
-      </c>
-      <c r="F27" s="11">
-        <v>0</v>
-      </c>
-      <c r="G27" s="11">
-        <v>0</v>
-      </c>
-      <c r="H27" s="11">
-        <v>0</v>
-      </c>
-      <c r="I27" s="13">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="J27" s="13">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="K27" s="13">
-        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data(Gerencia): poner al dia los Excel de oficial con el corte hasta agosto
Se habian quedado atras seis archivos cuando se corrigio el despliegue de
oficial trayendolo desde main: COMPRAS, INVENTARIO, INVENTARIO POR MESES,
TALENTO HUMANO, datos y VENTAS. pruebas/ ya estaba al dia.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/oficial/Gerencia/TALENTO HUMANO.xlsx
+++ b/oficial/Gerencia/TALENTO HUMANO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/APP OPAUSTRO/APP OPAUSTRO/Gerencia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{996977CD-B87C-4485-A8E4-AA98CA6C457C}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{674EB762-6582-42B0-8157-783A31CCBF6F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TALENTO ACTUAL" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="78">
   <si>
     <t>TALENTO HUMANO - SITUACION ACTUAL POR DEPARTAMENTO</t>
   </si>
@@ -266,6 +266,9 @@
   </si>
   <si>
     <t>Adulteracion de recibo de cobro</t>
+  </si>
+  <si>
+    <t>AGOSTO</t>
   </si>
 </sst>
 </file>
@@ -838,7 +841,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="16">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="C4" s="4">
         <v>79</v>
@@ -881,7 +884,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="16">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="C5" s="4">
         <v>22</v>
@@ -924,7 +927,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="16">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="C6" s="4">
         <v>29</v>
@@ -1020,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1893,6 +1896,120 @@
       </c>
       <c r="K24" s="13">
         <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="11">
+        <v>75</v>
+      </c>
+      <c r="E25" s="11">
+        <v>4</v>
+      </c>
+      <c r="F25" s="11">
+        <v>5</v>
+      </c>
+      <c r="G25" s="11">
+        <v>0</v>
+      </c>
+      <c r="H25" s="11">
+        <v>0</v>
+      </c>
+      <c r="I25" s="13">
+        <f t="shared" ref="I25:I27" si="9">IF(D25=0,0,(E25+F25)/D25)</f>
+        <v>0.12</v>
+      </c>
+      <c r="J25" s="13">
+        <f t="shared" ref="J25:J27" si="10">IF(D25=0,0,E25/D25)</f>
+        <v>5.3333333333333337E-2</v>
+      </c>
+      <c r="K25" s="13">
+        <f t="shared" ref="K25:K27" si="11">IF(D25=0,0,F25/D25)</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="11">
+        <v>22</v>
+      </c>
+      <c r="E26" s="11">
+        <v>0</v>
+      </c>
+      <c r="F26" s="11">
+        <v>0</v>
+      </c>
+      <c r="G26" s="11">
+        <v>0</v>
+      </c>
+      <c r="H26" s="11">
+        <v>0</v>
+      </c>
+      <c r="I26" s="13">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J26" s="13">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="K26" s="13">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="11">
+        <v>29</v>
+      </c>
+      <c r="E27" s="11">
+        <v>0</v>
+      </c>
+      <c r="F27" s="11">
+        <v>0</v>
+      </c>
+      <c r="G27" s="11">
+        <v>0</v>
+      </c>
+      <c r="H27" s="11">
+        <v>0</v>
+      </c>
+      <c r="I27" s="13">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="13">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="K27" s="13">
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>